<commit_message>
Add Zhuanzhuan platform section
</commit_message>
<xml_diff>
--- a/iphone16pm-512g-report-2026-09-04.xlsx
+++ b/iphone16pm-512g-report-2026-09-04.xlsx
@@ -12,14 +12,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="结论" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成色报价" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="平台检索" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本对比" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验机清单" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源链接" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="转转平台" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本对比" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验机清单" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源链接" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'实时单机库存'!$A$4:$S$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'平台检索'!$A$4:$Q$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'来源链接'!$A$4:$F$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'来源链接'!$A$4:$F$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +31,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="¥#,##0"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -150,8 +151,35 @@
       <color rgb="001769F2"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <color rgb="0044546A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <color rgb="001F2937"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <color rgb="001769E0"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -248,8 +276,23 @@
         <fgColor rgb="00FFF0F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001769E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F75B5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F8FD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -378,12 +421,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E2F3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -563,6 +611,24 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4489,22 +4555,22 @@
       </c>
       <c r="K11" s="21" t="inlineStr">
         <is>
-          <t>公开网页未取得当日目标机价和完整同机报告</t>
+          <t>官方介绍称官方验商品一物一验并输出详细报告；公开网页未取得9/4目标单机价格/同机报告</t>
         </is>
       </c>
       <c r="L11" s="21" t="inlineStr">
         <is>
-          <t>以App商品页为准</t>
+          <t>官方介绍称官方验手机支持7天无理由和专业质保；最终以下单页条款为准</t>
         </is>
       </c>
       <c r="M11" s="60" t="inlineStr">
         <is>
-          <t>报告完整后再买</t>
+          <t>值得蹲守，暂无可直接核价样本</t>
         </is>
       </c>
       <c r="N11" s="21" t="inlineStr">
         <is>
-          <t>保存同机报告、验机视频与退货条款</t>
+          <t>App筛国行A3297/512G/95新以上/白或原色；≤¥7300优先；保存同机报告和验机视频</t>
         </is>
       </c>
       <c r="O11" s="21" t="inlineStr">
@@ -4514,7 +4580,7 @@
       </c>
       <c r="P11" s="21" t="inlineStr">
         <is>
-          <t>平台名不是全原证明</t>
+          <t>今日无可公开核验的一机一价，不能硬报实时价</t>
         </is>
       </c>
       <c r="Q11" s="62" t="inlineStr">
@@ -5389,6 +5455,250 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="64" t="inlineStr">
+        <is>
+          <t>转转官方验｜iPhone 16 Pro Max 512G 专项筛选</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="65" t="inlineStr">
+        <is>
+          <t>公开核验快照：2026-09-04 08:39（中国标准时间）｜转转值得蹲守，但平台名和“官方验”都不能自动证明全原无拆</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B4" s="66" t="inlineStr">
+        <is>
+          <t>9/4核验结果</t>
+        </is>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>证据等级</t>
+        </is>
+      </c>
+      <c r="D4" s="66" t="inlineStr">
+        <is>
+          <t>购机动作</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="67" t="inlineStr">
+        <is>
+          <t>当天目标机价格</t>
+        </is>
+      </c>
+      <c r="B5" s="67" t="inlineStr">
+        <is>
+          <t>公开网页端未取得国行A3297/512G/95新以上的一机一价和完整同机报告</t>
+        </is>
+      </c>
+      <c r="C5" s="67" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D5" s="67" t="inlineStr">
+        <is>
+          <t>转转App内重新搜索，不把搜索摘要或平台均价当实时报价</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="68" t="inlineStr">
+        <is>
+          <t>官方验能力</t>
+        </is>
+      </c>
+      <c r="B6" s="68" t="inlineStr">
+        <is>
+          <t>官方介绍：官方验商品一物一验，由真人质检并输出详细质检报告</t>
+        </is>
+      </c>
+      <c r="C6" s="68" t="inlineStr">
+        <is>
+          <t>A（平台自述）</t>
+        </is>
+      </c>
+      <c r="D6" s="68" t="inlineStr">
+        <is>
+          <t>只看同机报告；逐项对上商品编号、容量、颜色、电池和外观照片</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>退换与质保</t>
+        </is>
+      </c>
+      <c r="B7" s="67" t="inlineStr">
+        <is>
+          <t>官方介绍：官方验手机支持7天无理由退货和专业质保；具体范围可能随订单变化</t>
+        </is>
+      </c>
+      <c r="C7" s="67" t="inlineStr">
+        <is>
+          <t>A（平台自述）</t>
+        </is>
+      </c>
+      <c r="D7" s="67" t="inlineStr">
+        <is>
+          <t>付款前截图订单页的退货条件、质保范围和运费责任</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="68" t="inlineStr">
+        <is>
+          <t>推荐筛选</t>
+        </is>
+      </c>
+      <c r="B8" s="68" t="inlineStr">
+        <is>
+          <t>国行A3297、512G、95新以上、白色/原色、原厂电池≥90%；高价机建议≥95%</t>
+        </is>
+      </c>
+      <c r="C8" s="68" t="inlineStr">
+        <is>
+          <t>购机标准</t>
+        </is>
+      </c>
+      <c r="D8" s="68" t="inlineStr">
+        <is>
+          <t>≤¥7300优先；¥7301–7500只在电池≥95%且报告完整时考虑</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="67" t="inlineStr">
+        <is>
+          <t>必须过的报告项</t>
+        </is>
+      </c>
+      <c r="B9" s="67" t="inlineStr">
+        <is>
+          <t>部件与维修历史、屏幕、Face ID、摄像头、进水、主板、螺丝/缝隙、原厂电池和循环次数</t>
+        </is>
+      </c>
+      <c r="C9" s="67" t="inlineStr">
+        <is>
+          <t>硬门槛</t>
+        </is>
+      </c>
+      <c r="D9" s="67" t="inlineStr">
+        <is>
+          <t>任何“未知部件”、功能异常、资源机、官换机、扩容、改卡或维修史不明都跳过</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="68" t="inlineStr">
+        <is>
+          <t>无拆无翻新证明</t>
+        </is>
+      </c>
+      <c r="B10" s="68" t="inlineStr">
+        <is>
+          <t>转转报告可降低风险，但公开页面未提供能够独立证明“从未拆机”的目标单机证据</t>
+        </is>
+      </c>
+      <c r="C10" s="68" t="inlineStr">
+        <is>
+          <t>未证实</t>
+        </is>
+      </c>
+      <c r="D10" s="68" t="inlineStr">
+        <is>
+          <t>高价按“全原无拆”购买时，要求可追责书面承诺；必要时在退货期内专业拆检</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="67" t="inlineStr">
+        <is>
+          <t>交易留证</t>
+        </is>
+      </c>
+      <c r="B11" s="67" t="inlineStr">
+        <is>
+          <t>保存同机报告、商品照片、客服承诺、订单条款和完整开箱验机视频</t>
+        </is>
+      </c>
+      <c r="C11" s="67" t="inlineStr">
+        <is>
+          <t>必要</t>
+        </is>
+      </c>
+      <c r="D11" s="67" t="inlineStr">
+        <is>
+          <t>全程平台支付；不私聊转账；收货后先验机再迁移数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="A12" s="68" t="inlineStr">
+        <is>
+          <t>9/4结论</t>
+        </is>
+      </c>
+      <c r="B12" s="68" t="inlineStr">
+        <is>
+          <t>转转新增为独立优先筛选平台，但今天没有可公开核验的一机一价合格样本</t>
+        </is>
+      </c>
+      <c r="C12" s="68" t="inlineStr">
+        <is>
+          <t>谨慎推荐</t>
+        </is>
+      </c>
+      <c r="D12" s="68" t="inlineStr">
+        <is>
+          <t>可蹲守，不盲买；若App发现≤¥7300且报告完整的国行机，再与爱回收¥7290候选对比</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="69" t="inlineStr">
+        <is>
+          <t>官方入口：转转官网 https://www.zhuanzhuan.com/index.html ｜ App Store https://apps.apple.com/cn/app/id1002355194</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A15:D15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I9"/>
@@ -5725,7 +6035,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6236,7 +6546,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6968,12 +7278,34 @@
       </c>
     </row>
     <row r="27" ht="38" customHeight="1">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="62" t="n"/>
+      <c r="A27" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>转转官网</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>官方验平台入口；网页端未公开9/4目标单机价格和完整同机报告</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04 08:39（中国标准时间）</t>
+        </is>
+      </c>
+      <c r="F27" s="62" t="inlineStr">
+        <is>
+          <t>https://www.zhuanzhuan.com/index.html</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="38" customHeight="1">
       <c r="A28" s="3" t="n"/>
@@ -7028,11 +7360,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>